<commit_message>
Cleaning of pvol files before next date is processed
</commit_message>
<xml_diff>
--- a/output/batch_results.xlsx
+++ b/output/batch_results.xlsx
@@ -99276,6 +99276,174 @@
       <c r="Q1796"/>
       <c r="R1796"/>
     </row>
+    <row r="1797">
+      <c r="A1797" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1797" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1797" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1797" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1797" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1797" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1797" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1797" t="s">
+        <v>37</v>
+      </c>
+      <c r="I1797" t="n">
+        <v>329</v>
+      </c>
+      <c r="J1797" t="n">
+        <v>39.054721</v>
+      </c>
+      <c r="K1797" t="n">
+        <v>-77.10895</v>
+      </c>
+      <c r="L1797" t="n">
+        <v>39.278491</v>
+      </c>
+      <c r="M1797" t="n">
+        <v>-77.282069</v>
+      </c>
+      <c r="N1797" t="n">
+        <v>0.1586</v>
+      </c>
+      <c r="O1797" t="n">
+        <v>13</v>
+      </c>
+      <c r="P1797" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q1797" t="n">
+        <v>763.39</v>
+      </c>
+      <c r="R1797" t="n">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="1798">
+      <c r="A1798" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1798" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1798" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1798" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1798" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1798" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1798" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1798" t="s">
+        <v>43</v>
+      </c>
+      <c r="I1798" t="n">
+        <v>315</v>
+      </c>
+      <c r="J1798" t="n">
+        <v>39.053369</v>
+      </c>
+      <c r="K1798" t="n">
+        <v>-77.111169</v>
+      </c>
+      <c r="L1798" t="n">
+        <v>39.231468</v>
+      </c>
+      <c r="M1798" t="n">
+        <v>-77.340494</v>
+      </c>
+      <c r="N1798" t="n">
+        <v>0.1586</v>
+      </c>
+      <c r="O1798" t="n">
+        <v>14</v>
+      </c>
+      <c r="P1798" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q1798" t="n">
+        <v>582.48</v>
+      </c>
+      <c r="R1798" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="1799">
+      <c r="A1799" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1799" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1799" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1799" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1799" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1799" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1799" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1799" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1799" t="n">
+        <v>274</v>
+      </c>
+      <c r="J1799" t="n">
+        <v>39.047628</v>
+      </c>
+      <c r="K1799" t="n">
+        <v>-77.114523</v>
+      </c>
+      <c r="L1799" t="n">
+        <v>39.064743</v>
+      </c>
+      <c r="M1799" t="n">
+        <v>-77.437261</v>
+      </c>
+      <c r="N1799" t="n">
+        <v>0.1586</v>
+      </c>
+      <c r="O1799" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="P1799" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q1799" t="n">
+        <v>306.91</v>
+      </c>
+      <c r="R1799" t="n">
+        <v>1.18</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>